<commit_message>
Updated files for week 6 tutorial
</commit_message>
<xml_diff>
--- a/Documents/5EAttendance.xlsx
+++ b/Documents/5EAttendance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bayle\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baz/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66DC4E0E-5306-4463-BA93-96D6F20101A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC0338A-29EF-CC41-8098-A25C85CBCAD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{CB148301-9041-45AB-8343-A4789F54342C}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="34200" windowHeight="21440" xr2:uid="{CB148301-9041-45AB-8343-A4789F54342C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="19">
   <si>
     <t>P = Present, L = Late, E = Excused, U = Unexcused</t>
   </si>
@@ -87,6 +87,12 @@
   </si>
   <si>
     <t>Safia Farah - up2214501</t>
+  </si>
+  <si>
+    <t>Present</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P </t>
   </si>
 </sst>
 </file>
@@ -209,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -245,6 +251,17 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -581,13 +598,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C41EF30-CFB6-4C55-80FB-648F0AAE86D6}">
-  <dimension ref="A1:Z48"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AA48"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="24" max="26" width="15.5546875" customWidth="1"/>
+    <col min="24" max="26" width="15.5" customWidth="1"/>
+    <col min="27" max="27" width="8.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="12"/>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -618,8 +636,9 @@
       <c r="X1" s="12"/>
       <c r="Y1" s="12"/>
       <c r="Z1" s="12"/>
-    </row>
-    <row r="2" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA1" s="18"/>
+    </row>
+    <row r="2" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12"/>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -646,8 +665,9 @@
       <c r="X2" s="12"/>
       <c r="Y2" s="12"/>
       <c r="Z2" s="12"/>
-    </row>
-    <row r="3" spans="1:26" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA2" s="18"/>
+    </row>
+    <row r="3" spans="1:27" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
         <v>4</v>
       </c>
@@ -722,8 +742,11 @@
       <c r="Z3" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:26" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA3" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="14"/>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -816,236 +839,432 @@
       <c r="Z4" s="10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA4" s="16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" t="s">
-        <v>8</v>
-      </c>
+      <c r="D5" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
       <c r="X5" s="2">
         <f>COUNTIF(D5:W5,$X$4)</f>
         <v>0</v>
       </c>
       <c r="Y5" s="2">
         <f>COUNTIF(D5:W5,$Y$4)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z5" s="2">
         <f>COUNTIF(D5:W5,$Z$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA5" s="6">
+        <f>COUNTIF(D5:W5,"P")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
-      <c r="D6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" t="s">
-        <v>8</v>
-      </c>
+      <c r="D6" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
       <c r="X6" s="2">
         <f t="shared" ref="X6:X11" si="1">COUNTIF(D6:W6,$X5)</f>
         <v>0</v>
       </c>
       <c r="Y6" s="2">
         <f t="shared" ref="Y6:Y11" si="2">COUNTIF(D6:W6,$Y$4)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z6" s="2">
         <f t="shared" ref="Z6:Z11" si="3">COUNTIF(D6:W6,$Z$4)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="AA6" s="6">
+        <f t="shared" ref="AA6:AA11" si="4">COUNTIF(D6:W6,"P")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
-      <c r="D7" t="s">
+      <c r="D7" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" t="s">
-        <v>8</v>
-      </c>
+      <c r="E7" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="19"/>
       <c r="X7" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y7" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z7" s="2">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="AA7" s="6">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="D8" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F8" t="s">
-        <v>8</v>
-      </c>
+      <c r="F8" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
       <c r="X8" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y8" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z8" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="AA8" s="6">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
-      <c r="D9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="D9" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F9" t="s">
-        <v>8</v>
-      </c>
+      <c r="F9" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H9" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
       <c r="X9" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y9" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z9" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="6">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>14</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
-      <c r="D10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="D10" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="F10" t="s">
-        <v>8</v>
-      </c>
+      <c r="F10" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H10" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
+      <c r="U10" s="19"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19"/>
       <c r="X10" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y10" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z10" s="2">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="AA10" s="6">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
-      <c r="D11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="D11" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="F11" t="s">
-        <v>8</v>
-      </c>
+      <c r="F11" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H11" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="19"/>
+      <c r="Q11" s="19"/>
+      <c r="R11" s="19"/>
+      <c r="S11" s="19"/>
+      <c r="T11" s="19"/>
+      <c r="U11" s="19"/>
+      <c r="V11" s="19"/>
+      <c r="W11" s="19"/>
       <c r="X11" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y11" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z11" s="2">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="AA11" s="6">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
       <c r="X12" s="2"/>
       <c r="Y12" s="6"/>
-      <c r="Z12" s="4"/>
-    </row>
-    <row r="13" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Z12" s="17"/>
+      <c r="AA12" s="6"/>
+    </row>
+    <row r="13" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="X13" s="2"/>
       <c r="Y13" s="6"/>
-      <c r="Z13" s="4"/>
-    </row>
-    <row r="14" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Z13" s="17"/>
+      <c r="AA13" s="6"/>
+    </row>
+    <row r="14" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
       <c r="X14" s="2"/>
       <c r="Y14" s="6"/>
-      <c r="Z14" s="4"/>
-    </row>
-    <row r="15" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Z14" s="17"/>
+      <c r="AA14" s="6"/>
+    </row>
+    <row r="15" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
       <c r="X15" s="2"/>
       <c r="Y15" s="6"/>
-      <c r="Z15" s="4"/>
-    </row>
-    <row r="16" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Z15" s="17"/>
+      <c r="AA15" s="6"/>
+    </row>
+    <row r="16" spans="1:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
@@ -1053,7 +1272,7 @@
       <c r="Y16" s="6"/>
       <c r="Z16" s="4"/>
     </row>
-    <row r="17" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -1061,7 +1280,7 @@
       <c r="Y17" s="6"/>
       <c r="Z17" s="4"/>
     </row>
-    <row r="18" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="11"/>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -1069,7 +1288,7 @@
       <c r="Y18" s="6"/>
       <c r="Z18" s="4"/>
     </row>
-    <row r="19" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
@@ -1077,7 +1296,7 @@
       <c r="Y19" s="6"/>
       <c r="Z19" s="4"/>
     </row>
-    <row r="20" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11"/>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -1085,7 +1304,7 @@
       <c r="Y20" s="6"/>
       <c r="Z20" s="4"/>
     </row>
-    <row r="21" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="11"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -1093,7 +1312,7 @@
       <c r="Y21" s="6"/>
       <c r="Z21" s="4"/>
     </row>
-    <row r="22" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="11"/>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
@@ -1101,7 +1320,7 @@
       <c r="Y22" s="6"/>
       <c r="Z22" s="4"/>
     </row>
-    <row r="23" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="11"/>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
@@ -1109,7 +1328,7 @@
       <c r="Y23" s="6"/>
       <c r="Z23" s="4"/>
     </row>
-    <row r="24" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="11"/>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
@@ -1117,7 +1336,7 @@
       <c r="Y24" s="6"/>
       <c r="Z24" s="4"/>
     </row>
-    <row r="25" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -1125,7 +1344,7 @@
       <c r="Y25" s="6"/>
       <c r="Z25" s="4"/>
     </row>
-    <row r="26" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="11"/>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
@@ -1133,7 +1352,7 @@
       <c r="Y26" s="6"/>
       <c r="Z26" s="4"/>
     </row>
-    <row r="27" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="11"/>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
@@ -1141,7 +1360,7 @@
       <c r="Y27" s="6"/>
       <c r="Z27" s="4"/>
     </row>
-    <row r="28" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="11"/>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
@@ -1149,7 +1368,7 @@
       <c r="Y28" s="6"/>
       <c r="Z28" s="4"/>
     </row>
-    <row r="29" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="11"/>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -1157,7 +1376,7 @@
       <c r="Y29" s="6"/>
       <c r="Z29" s="4"/>
     </row>
-    <row r="30" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="11"/>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -1165,7 +1384,7 @@
       <c r="Y30" s="6"/>
       <c r="Z30" s="4"/>
     </row>
-    <row r="31" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="11"/>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
@@ -1173,7 +1392,7 @@
       <c r="Y31" s="6"/>
       <c r="Z31" s="4"/>
     </row>
-    <row r="32" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="11"/>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
@@ -1181,7 +1400,7 @@
       <c r="Y32" s="6"/>
       <c r="Z32" s="4"/>
     </row>
-    <row r="33" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="11"/>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
@@ -1189,7 +1408,7 @@
       <c r="Y33" s="6"/>
       <c r="Z33" s="4"/>
     </row>
-    <row r="34" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="11"/>
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
@@ -1197,7 +1416,7 @@
       <c r="Y34" s="6"/>
       <c r="Z34" s="4"/>
     </row>
-    <row r="35" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="11"/>
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
@@ -1205,7 +1424,7 @@
       <c r="Y35" s="6"/>
       <c r="Z35" s="4"/>
     </row>
-    <row r="36" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="11"/>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
@@ -1213,7 +1432,7 @@
       <c r="Y36" s="6"/>
       <c r="Z36" s="4"/>
     </row>
-    <row r="37" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="11"/>
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
@@ -1221,7 +1440,7 @@
       <c r="Y37" s="6"/>
       <c r="Z37" s="4"/>
     </row>
-    <row r="38" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="11"/>
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
@@ -1229,7 +1448,7 @@
       <c r="Y38" s="6"/>
       <c r="Z38" s="4"/>
     </row>
-    <row r="39" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="11"/>
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
@@ -1237,7 +1456,7 @@
       <c r="Y39" s="6"/>
       <c r="Z39" s="4"/>
     </row>
-    <row r="40" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="11"/>
       <c r="B40" s="11"/>
       <c r="C40" s="11"/>
@@ -1245,7 +1464,7 @@
       <c r="Y40" s="6"/>
       <c r="Z40" s="4"/>
     </row>
-    <row r="41" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="11"/>
       <c r="B41" s="11"/>
       <c r="C41" s="11"/>
@@ -1253,7 +1472,7 @@
       <c r="Y41" s="6"/>
       <c r="Z41" s="4"/>
     </row>
-    <row r="42" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="11"/>
       <c r="B42" s="11"/>
       <c r="C42" s="11"/>
@@ -1261,7 +1480,7 @@
       <c r="Y42" s="6"/>
       <c r="Z42" s="4"/>
     </row>
-    <row r="43" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="11"/>
       <c r="B43" s="11"/>
       <c r="C43" s="11"/>
@@ -1269,7 +1488,7 @@
       <c r="Y43" s="6"/>
       <c r="Z43" s="4"/>
     </row>
-    <row r="44" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="11"/>
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
@@ -1277,7 +1496,7 @@
       <c r="Y44" s="6"/>
       <c r="Z44" s="4"/>
     </row>
-    <row r="45" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="11"/>
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
@@ -1285,7 +1504,7 @@
       <c r="Y45" s="6"/>
       <c r="Z45" s="4"/>
     </row>
-    <row r="46" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="11"/>
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
@@ -1293,7 +1512,7 @@
       <c r="Y46" s="6"/>
       <c r="Z46" s="4"/>
     </row>
-    <row r="47" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="11"/>
       <c r="B47" s="11"/>
       <c r="C47" s="11"/>
@@ -1301,7 +1520,7 @@
       <c r="Y47" s="6"/>
       <c r="Z47" s="4"/>
     </row>
-    <row r="48" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="11"/>
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
@@ -1311,6 +1530,38 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="A3:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="Q1:Z2"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A46:C46"/>
     <mergeCell ref="A47:C47"/>
@@ -1327,38 +1578,6 @@
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A16:C16"/>
-    <mergeCell ref="Q1:Z2"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="A3:C4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>